<commit_message>
Add low cable EZ bar curl image mapping
</commit_message>
<xml_diff>
--- a/docs/assets/gymflow_liikepankki_kuvat_en.xlsx
+++ b/docs/assets/gymflow_liikepankki_kuvat_en.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/053365cd39567d92/Ohjelmointi_projektit/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/053365cd39567d92/Ohjelmointi_projektit/gymflow-dashboard/docs/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_A3B845323DEF4608EFC24119799D8980AB197199" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="14_{AB726984-C1AA-4B77-B17B-B40D447984E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C4636C5-6EF4-429E-9640-2F85C1EA8196}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-810" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="167">
   <si>
     <t>#</t>
   </si>
@@ -526,6 +526,15 @@
   </si>
   <si>
     <t>Määrä</t>
+  </si>
+  <si>
+    <t>Hauiskääntö alataljassa</t>
+  </si>
+  <si>
+    <t>low-cable-ez-bar-curl.png</t>
+  </si>
+  <si>
+    <t>Low Cable EZ Bar Curl</t>
   </si>
 </sst>
 </file>
@@ -605,7 +614,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -634,6 +643,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -905,7 +917,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ExerciseImageList" displayName="ExerciseImageList" ref="A1:F48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ExerciseImageList" displayName="ExerciseImageList" ref="A1:F49">
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="#"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Kategoria"/>
@@ -1067,7 +1079,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1203,16 +1215,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>26</v>
+        <v>91</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>10</v>
@@ -1223,16 +1235,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>28</v>
+        <v>93</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>29</v>
+        <v>94</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>30</v>
+        <v>95</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>10</v>
@@ -1243,16 +1255,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>31</v>
+        <v>164</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>33</v>
+        <v>166</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>165</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>10</v>
@@ -1266,13 +1278,13 @@
         <v>24</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>10</v>
@@ -1283,16 +1295,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>10</v>
@@ -1303,16 +1315,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>10</v>
@@ -1323,16 +1335,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>10</v>
@@ -1346,13 +1358,13 @@
         <v>37</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>10</v>
@@ -1366,13 +1378,13 @@
         <v>37</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>10</v>
@@ -1386,13 +1398,13 @@
         <v>37</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>10</v>
@@ -1403,16 +1415,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>10</v>
@@ -1423,16 +1435,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>10</v>
@@ -1443,16 +1455,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>10</v>
@@ -1463,16 +1475,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>10</v>
@@ -1483,16 +1495,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>10</v>
@@ -1503,16 +1515,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>10</v>
@@ -1523,16 +1535,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>10</v>
@@ -1543,16 +1555,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>10</v>
@@ -1566,13 +1578,13 @@
         <v>73</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>10</v>
@@ -1583,16 +1595,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>10</v>
@@ -1603,16 +1615,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>10</v>
@@ -1623,16 +1635,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>10</v>
@@ -1643,16 +1655,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>10</v>
@@ -1666,13 +1678,13 @@
         <v>96</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>10</v>
@@ -1683,16 +1695,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>24</v>
+        <v>96</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>10</v>
@@ -1706,13 +1718,13 @@
         <v>24</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>10</v>
@@ -1723,16 +1735,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>10</v>
@@ -1746,13 +1758,13 @@
         <v>37</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>10</v>
@@ -1766,13 +1778,13 @@
         <v>37</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F35" s="4" t="s">
         <v>10</v>
@@ -1783,16 +1795,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>10</v>
@@ -1806,13 +1818,13 @@
         <v>63</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>10</v>
@@ -1826,13 +1838,13 @@
         <v>63</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>10</v>
@@ -1843,16 +1855,16 @@
         <v>38</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>10</v>
@@ -1866,13 +1878,13 @@
         <v>73</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>10</v>
@@ -1886,13 +1898,13 @@
         <v>73</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>10</v>
@@ -1906,13 +1918,13 @@
         <v>73</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>10</v>
@@ -1923,16 +1935,16 @@
         <v>42</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>10</v>
@@ -1946,13 +1958,13 @@
         <v>86</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F44" s="4" t="s">
         <v>10</v>
@@ -1966,13 +1978,13 @@
         <v>86</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>10</v>
@@ -1986,13 +1998,13 @@
         <v>86</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="F46" s="4" t="s">
         <v>10</v>
@@ -2006,13 +2018,13 @@
         <v>86</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>10</v>
@@ -2026,20 +2038,40 @@
         <v>86</v>
       </c>
       <c r="C48" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="21.95" customHeight="1">
+      <c r="A49" s="4">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="D48" s="5" t="s">
+      <c r="D49" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E48" s="5" t="s">
+      <c r="E49" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="F48" s="4" t="s">
+      <c r="F49" s="4" t="s">
         <v>10</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F48">
+  <conditionalFormatting sqref="F2:F49">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>F2="x"</formula>
     </cfRule>

</xml_diff>